<commit_message>
update soccer prediction app
</commit_message>
<xml_diff>
--- a/output/elite_predictions.xlsx
+++ b/output/elite_predictions.xlsx
@@ -486,17 +486,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>USL League Two</t>
+          <t>USL Championship</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Dothan United</t>
+          <t>Birmingham Legion</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Birmingham Legion II</t>
+          <t>Louisville City</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -526,12 +526,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>4-0</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>WON</t>
+          <t>LOST</t>
         </is>
       </c>
       <c r="L2" t="n">
@@ -541,37 +541,37 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>I Liga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Chrobry Głogów</t>
+          <t>HLM</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>ŁKS Łódź</t>
+          <t>Pikine</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -581,12 +581,12 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>HOME WIN</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -601,52 +601,52 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Regionalliga - Promotion Play-offs</t>
+          <t>Ettan - Södra</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Lokomotive Leipzig</t>
+          <t>Laholm</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Würzburger Kickers</t>
+          <t>Hässleholms IF</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t>2-3</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>OVER 2.5</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>AWAY WIN</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
           <t>1-2</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>OVER 2.5</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>AWAY WIN</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>0-1</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -661,27 +661,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Kvindeliga</t>
+          <t>Division 2 - Norra Götaland</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>KoldingQ W</t>
+          <t>Stenungsund</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Fortuna Hjørring W</t>
+          <t>Vänersborgs IF</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -701,17 +701,17 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>AWAY WIN</t>
+          <t>DRAW</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>5-0</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>WON</t>
+          <t>LOST</t>
         </is>
       </c>
       <c r="L5" t="n">
@@ -721,27 +721,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Regionalliga - Ost</t>
+          <t>3. Division</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Traiskirchen</t>
+          <t>Sundby</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Neusiedl</t>
+          <t>Holbæk B&amp;I</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -766,7 +766,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2-4</t>
+          <t>1-5</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -781,27 +781,27 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kuwait</t>
+          <t>World</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>Friendlies</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Al Fahaheel</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Al Salmiyah</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>3-3</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -821,12 +821,12 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>HOME WIN</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>0-2</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -846,27 +846,27 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CAF Cup of Nations - U17</t>
+          <t>Friendlies</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Egypt U17</t>
+          <t>Andorra</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Tanzania U17</t>
+          <t>Liechtenstein</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -876,7 +876,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>OVER 2.5</t>
+          <t>UNDER 2.5</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
@@ -886,12 +886,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>0-0</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>LOST</t>
+          <t>WON</t>
         </is>
       </c>
       <c r="L8" t="n">
@@ -901,27 +901,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>World</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>UEFA U17 Championship</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Estonia U17</t>
+          <t>AS Camberene</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Croatia U17</t>
+          <t>Jaraaf</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0-3</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -936,22 +936,22 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>OVER 2.5</t>
+          <t>UNDER 2.5</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>AWAY WIN</t>
+          <t>HOME WIN</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>0-2</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>WON</t>
+          <t>LOST</t>
         </is>
       </c>
       <c r="L9" t="n">
@@ -961,57 +961,57 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Esiliiga B</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tulevik</t>
+          <t>Casa Sport</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Parnu JK Vaprus U21</t>
+          <t>DSC</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>0-0</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>OVER 2.5</t>
+          <t>UNDER 2.5</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>HOME WIN</t>
+          <t>DRAW</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>3-1</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>WON</t>
+          <t>LOST</t>
         </is>
       </c>
       <c r="L10" t="n">
@@ -1021,27 +1021,27 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>World</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Esiliiga B</t>
+          <t>Friendlies</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Narva U21</t>
+          <t>Iran</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Johvi Phoenix</t>
+          <t>Mali</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>5-1</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1056,17 +1056,17 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>OVER 2.5</t>
+          <t>UNDER 2.5</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>HOME WIN</t>
+          <t>DRAW</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -1081,32 +1081,32 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Esiliiga A</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Tartu Welco</t>
+          <t>Génération Foot</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Nõmme Kalju II</t>
+          <t>AJEL</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>4-0</t>
+          <t>3-1</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1126,12 +1126,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>WON</t>
+          <t>LOST</t>
         </is>
       </c>
       <c r="L12" t="n">
@@ -1141,27 +1141,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Esiliiga A</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>FCI Levadia II</t>
+          <t>Guédiawaye</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Elva</t>
+          <t>Teungueth</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>2-2</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -1181,12 +1181,12 @@
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>HOME WIN</t>
+          <t>DRAW</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1-3</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -1201,57 +1201,57 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Esiliiga A</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>FC Tallinn</t>
+          <t>La Linguère</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Maardu</t>
+          <t>Wally Daan</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
+          <t>4-2</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>OVER 2.5</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>HOME WIN</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
           <t>1-1</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>UNDER 2.5</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>DRAW</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>0-0</t>
-        </is>
-      </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>WON</t>
+          <t>LOST</t>
         </is>
       </c>
       <c r="L14" t="n">
@@ -1261,42 +1261,42 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Georgia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Erovnuli Liga</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Torpedo Kutaisi</t>
+          <t>Ouakam</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Gagra</t>
+          <t>Sonacos</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>OVER 2.5</t>
+          <t>UNDER 2.5</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -1306,12 +1306,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>WON</t>
+          <t>LOST</t>
         </is>
       </c>
       <c r="L15" t="n">
@@ -1321,32 +1321,32 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Esiliiga B</t>
+          <t>Ligue 1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tallinna Kalev II</t>
+          <t>Gorée</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Luunja</t>
+          <t>Stade de Mbour</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>3-2</t>
+          <t>0-8</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1361,12 +1361,12 @@
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>HOME WIN</t>
+          <t>AWAY WIN</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>0-1</t>
+          <t>0-0</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -1381,32 +1381,32 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>World</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>First League</t>
+          <t>UEFA U17 Championship</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Septemvri Sofia</t>
+          <t>Italy U17</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Yantra 2019</t>
+          <t>Spain U17</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>3-0</t>
+          <t>3-2</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1426,12 +1426,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>WON</t>
+          <t>LOST</t>
         </is>
       </c>
       <c r="L17" t="n">
@@ -1441,27 +1441,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>World</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ykkönen</t>
+          <t>Friendlies Women</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>JJK</t>
+          <t>Sweden U18 W</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>OLS</t>
+          <t>Norway U18 W</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>2-3</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -1476,17 +1476,17 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>UNDER 2.5</t>
+          <t>OVER 2.5</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>AWAY WIN</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -1501,32 +1501,32 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Mali</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Ykkönen</t>
+          <t>Première Division</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>FC jazz</t>
+          <t>USFAS Bamako</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>SalPa</t>
+          <t>Onze Créateurs</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>4-2</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1536,7 +1536,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>OVER 2.5</t>
+          <t>UNDER 2.5</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -1546,12 +1546,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>3-0</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>LOST</t>
+          <t>WON</t>
         </is>
       </c>
       <c r="L19" t="n">
@@ -1561,42 +1561,42 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Sweden</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Iraqi League</t>
+          <t>Division 2 - Södra Götaland</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Naft Maysan</t>
+          <t>Sölvesborg</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Al Quwa Al Jawiya</t>
+          <t>Torns</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>3-1</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>OVER 2.5</t>
+          <t>UNDER 2.5</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -1606,7 +1606,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>0-2</t>
+          <t>1-3</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -1621,32 +1621,32 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>World</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Iraqi League</t>
+          <t>Friendlies</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Al Minaa Basra</t>
+          <t>Afghanistan</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Al Talaba</t>
+          <t>Bangladesh U23</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1656,17 +1656,17 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>OVER 2.5</t>
+          <t>UNDER 2.5</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>AWAY WIN</t>
+          <t>HOME WIN</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>1-1</t>
+          <t>0-0</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -1681,32 +1681,32 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>World</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Iraqi League</t>
+          <t>Friendlies Women</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Al Karkh</t>
+          <t>Germany U23 W</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Al Shorta</t>
+          <t>Denmark U23 W</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>2-1</t>
+          <t>0-4</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1721,12 +1721,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>HOME WIN</t>
+          <t>AWAY WIN</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>0-2</t>
+          <t>2-0</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -1741,32 +1741,32 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Belarus</t>
+          <t>World</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Coppa</t>
+          <t>Friendlies</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Viktoriya Maryina Horka</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Nadezhda</t>
+          <t>Cyprus</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>NO</t>
+          <t>YES</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1776,22 +1776,22 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>UNDER 2.5</t>
+          <t>OVER 2.5</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>HOME WIN</t>
+          <t>AWAY WIN</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>1-0</t>
+          <t>1-1</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>WON</t>
+          <t>LOST</t>
         </is>
       </c>
       <c r="L23" t="n">
@@ -1801,27 +1801,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Belarus</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Coppa</t>
+          <t>Kakkonen - Lohko A</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tekhnolog</t>
+          <t>PEPO</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Slonim</t>
+          <t>Reipas</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>3-1</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -1846,12 +1846,12 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>0-6</t>
+          <t>2-1</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>LOST</t>
+          <t>WON</t>
         </is>
       </c>
       <c r="L24" t="n">
@@ -1861,27 +1861,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Belarus</t>
+          <t>World</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Coppa</t>
+          <t>Friendlies</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DYuSSh-3 Pinsk</t>
+          <t>Northern Ireland</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>NFK Minsk</t>
+          <t>Guinea</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>2-0</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -1891,7 +1891,7 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -1901,12 +1901,12 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>HOME WIN</t>
+          <t>AWAY WIN</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>1-4</t>
+          <t>1-0</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -1921,27 +1921,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Ethiopia</t>
+          <t>World</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Premier League</t>
+          <t>Friendlies</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Mekelakeya</t>
+          <t>Burundi</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Arba Minch Kenema</t>
+          <t>Equatorial Guinea</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>0-2</t>
+          <t>0-1</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -1951,7 +1951,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>YES</t>
+          <t>NO</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1966,12 +1966,12 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>1-2</t>
+          <t>Not Played</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>WON</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="L26" t="n">

</xml_diff>